<commit_message>
split the proteome into five groupings and give each grouping its own runner
</commit_message>
<xml_diff>
--- a/02_Groups/HRvLR/c_data/study_groups.xlsx
+++ b/02_Groups/HRvLR/c_data/study_groups.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="186">
   <si>
     <t>sheet</t>
   </si>
@@ -369,12 +369,6 @@
   </si>
   <si>
     <t>0.5.9</t>
-  </si>
-  <si>
-    <t>htmlwidgets</t>
-  </si>
-  <si>
-    <t>1.6.4</t>
   </si>
   <si>
     <t>IRanges</t>
@@ -1520,7 +1514,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1850,7 +1844,7 @@
         <v>118</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1861,7 +1855,7 @@
         <v>120</v>
       </c>
       <c r="C31" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1902,7 +1896,7 @@
         <v>127</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="C35" t="s">
         <v>65</v>
@@ -1910,10 +1904,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
+        <v>128</v>
+      </c>
+      <c r="B36" t="s">
         <v>129</v>
-      </c>
-      <c r="B36" t="s">
-        <v>93</v>
       </c>
       <c r="C36" t="s">
         <v>65</v>
@@ -2048,18 +2042,18 @@
         <v>153</v>
       </c>
       <c r="C48" t="s">
-        <v>65</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B49" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C49" t="s">
-        <v>156</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -2081,7 +2075,7 @@
         <v>160</v>
       </c>
       <c r="C51" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -2092,7 +2086,7 @@
         <v>162</v>
       </c>
       <c r="C52" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -2144,7 +2138,7 @@
         <v>171</v>
       </c>
       <c r="B57" t="s">
-        <v>172</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
         <v>65</v>
@@ -2152,10 +2146,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
+        <v>172</v>
+      </c>
+      <c r="B58" t="s">
         <v>173</v>
-      </c>
-      <c r="B58" t="s">
-        <v>91</v>
       </c>
       <c r="C58" t="s">
         <v>65</v>
@@ -2224,17 +2218,6 @@
         <v>185</v>
       </c>
       <c r="C64" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" t="s">
-        <v>186</v>
-      </c>
-      <c r="B65" t="s">
-        <v>187</v>
-      </c>
-      <c r="C65" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>